<commit_message>
not perfect, just backup
</commit_message>
<xml_diff>
--- a/Data/Ecoli_phenotypes/fluxomics_datasets_gerosa.xlsx
+++ b/Data/Ecoli_phenotypes/fluxomics_datasets_gerosa.xlsx
@@ -290,9 +290,9 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E305"/>
-  <sheetFormatPr defaultColWidth="8.6875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6875" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -309,7 +309,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
         <v>5</v>
       </c>
@@ -317,7 +317,7 @@
         <v>6</v>
       </c>
       <c r="C2" s="0" t="n">
-        <v>13.584</v>
+        <v>-13.584</v>
       </c>
       <c r="D2" s="0" t="n">
         <v>0.29</v>
@@ -326,7 +326,7 @@
         <v>13.584</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
         <v>7</v>
       </c>
@@ -343,7 +343,7 @@
         <v>13.584</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
         <v>8</v>
       </c>
@@ -360,7 +360,7 @@
         <v>13.584</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
         <v>9</v>
       </c>
@@ -377,7 +377,7 @@
         <v>13.584</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
         <v>10</v>
       </c>
@@ -394,7 +394,7 @@
         <v>13.584</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
         <v>11</v>
       </c>
@@ -411,7 +411,7 @@
         <v>13.584</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
         <v>12</v>
       </c>
@@ -428,7 +428,7 @@
         <v>13.584</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
         <v>13</v>
       </c>
@@ -445,7 +445,7 @@
         <v>13.584</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
         <v>14</v>
       </c>
@@ -462,7 +462,7 @@
         <v>13.584</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
         <v>15</v>
       </c>
@@ -479,7 +479,7 @@
         <v>13.584</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
         <v>16</v>
       </c>
@@ -496,7 +496,7 @@
         <v>13.584</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
         <v>17</v>
       </c>
@@ -513,7 +513,7 @@
         <v>13.584</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
         <v>18</v>
       </c>
@@ -530,7 +530,7 @@
         <v>13.584</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
         <v>19</v>
       </c>
@@ -547,7 +547,7 @@
         <v>13.584</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
         <v>20</v>
       </c>
@@ -564,7 +564,7 @@
         <v>13.584</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
         <v>21</v>
       </c>
@@ -581,7 +581,7 @@
         <v>13.584</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
         <v>22</v>
       </c>
@@ -598,7 +598,7 @@
         <v>13.584</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
         <v>23</v>
       </c>
@@ -615,7 +615,7 @@
         <v>13.584</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
         <v>24</v>
       </c>
@@ -632,7 +632,7 @@
         <v>13.584</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="0" t="s">
         <v>25</v>
       </c>
@@ -649,7 +649,7 @@
         <v>13.584</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="0" t="s">
         <v>26</v>
       </c>
@@ -666,7 +666,7 @@
         <v>13.584</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="0" t="s">
         <v>27</v>
       </c>
@@ -683,7 +683,7 @@
         <v>13.584</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="0" t="s">
         <v>28</v>
       </c>
@@ -700,7 +700,7 @@
         <v>13.584</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="0" t="s">
         <v>29</v>
       </c>
@@ -717,7 +717,7 @@
         <v>13.584</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="0" t="s">
         <v>30</v>
       </c>
@@ -734,7 +734,7 @@
         <v>13.584</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="0" t="s">
         <v>31</v>
       </c>
@@ -751,7 +751,7 @@
         <v>13.584</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="0" t="s">
         <v>32</v>
       </c>
@@ -768,7 +768,7 @@
         <v>13.584</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="0" t="s">
         <v>33</v>
       </c>
@@ -785,7 +785,7 @@
         <v>13.584</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="0" t="s">
         <v>34</v>
       </c>
@@ -802,7 +802,7 @@
         <v>13.584</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="0" t="s">
         <v>35</v>
       </c>
@@ -819,7 +819,7 @@
         <v>13.584</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="0" t="s">
         <v>36</v>
       </c>
@@ -836,7 +836,7 @@
         <v>13.584</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="0" t="s">
         <v>37</v>
       </c>
@@ -853,7 +853,7 @@
         <v>13.584</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="0" t="s">
         <v>38</v>
       </c>
@@ -870,7 +870,7 @@
         <v>13.584</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="0" t="s">
         <v>39</v>
       </c>
@@ -887,7 +887,7 @@
         <v>13.584</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="0" t="s">
         <v>40</v>
       </c>
@@ -904,7 +904,7 @@
         <v>13.584</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="0" t="s">
         <v>41</v>
       </c>
@@ -921,7 +921,7 @@
         <v>13.584</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="0" t="s">
         <v>42</v>
       </c>
@@ -938,7 +938,7 @@
         <v>13.584</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="0" t="s">
         <v>43</v>
       </c>
@@ -955,7 +955,7 @@
         <v>13.584</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="0" t="s">
         <v>5</v>
       </c>
@@ -963,7 +963,7 @@
         <v>44</v>
       </c>
       <c r="C40" s="0" t="n">
-        <v>-3.32865961111111</v>
+        <v>3.32865961111111</v>
       </c>
       <c r="D40" s="0" t="n">
         <v>0.4924</v>
@@ -972,7 +972,7 @@
         <v>8.328</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="0" t="s">
         <v>7</v>
       </c>
@@ -980,7 +980,7 @@
         <v>44</v>
       </c>
       <c r="C41" s="0" t="n">
-        <v>8.328</v>
+        <v>-8.328</v>
       </c>
       <c r="D41" s="0" t="n">
         <v>0.4924</v>
@@ -989,7 +989,7 @@
         <v>8.328</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="0" t="s">
         <v>8</v>
       </c>
@@ -1006,7 +1006,7 @@
         <v>8.328</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="0" t="s">
         <v>9</v>
       </c>
@@ -1023,7 +1023,7 @@
         <v>8.328</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="0" t="s">
         <v>10</v>
       </c>
@@ -1040,7 +1040,7 @@
         <v>8.328</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="0" t="s">
         <v>11</v>
       </c>
@@ -1057,7 +1057,7 @@
         <v>8.328</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="0" t="s">
         <v>12</v>
       </c>
@@ -1074,7 +1074,7 @@
         <v>8.328</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="0" t="s">
         <v>13</v>
       </c>
@@ -1091,7 +1091,7 @@
         <v>8.328</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="0" t="s">
         <v>14</v>
       </c>
@@ -1108,7 +1108,7 @@
         <v>8.328</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="0" t="s">
         <v>15</v>
       </c>
@@ -1125,7 +1125,7 @@
         <v>8.328</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="0" t="s">
         <v>16</v>
       </c>
@@ -1142,7 +1142,7 @@
         <v>8.328</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="0" t="s">
         <v>17</v>
       </c>
@@ -1159,7 +1159,7 @@
         <v>8.328</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="0" t="s">
         <v>18</v>
       </c>
@@ -1176,7 +1176,7 @@
         <v>8.328</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="0" t="s">
         <v>19</v>
       </c>
@@ -1193,7 +1193,7 @@
         <v>8.328</v>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="0" t="s">
         <v>20</v>
       </c>
@@ -1210,7 +1210,7 @@
         <v>8.328</v>
       </c>
     </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="0" t="s">
         <v>21</v>
       </c>
@@ -1227,7 +1227,7 @@
         <v>8.328</v>
       </c>
     </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="0" t="s">
         <v>22</v>
       </c>
@@ -1244,7 +1244,7 @@
         <v>8.328</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="0" t="s">
         <v>23</v>
       </c>
@@ -1261,7 +1261,7 @@
         <v>8.328</v>
       </c>
     </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="0" t="s">
         <v>24</v>
       </c>
@@ -1278,7 +1278,7 @@
         <v>8.328</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="0" t="s">
         <v>25</v>
       </c>
@@ -1295,7 +1295,7 @@
         <v>8.328</v>
       </c>
     </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="60" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="0" t="s">
         <v>26</v>
       </c>
@@ -1312,7 +1312,7 @@
         <v>8.328</v>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="61" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="0" t="s">
         <v>27</v>
       </c>
@@ -1329,7 +1329,7 @@
         <v>8.328</v>
       </c>
     </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="0" t="s">
         <v>28</v>
       </c>
@@ -1346,7 +1346,7 @@
         <v>8.328</v>
       </c>
     </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="0" t="s">
         <v>29</v>
       </c>
@@ -1363,7 +1363,7 @@
         <v>8.328</v>
       </c>
     </row>
-    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="0" t="s">
         <v>30</v>
       </c>
@@ -1380,7 +1380,7 @@
         <v>8.328</v>
       </c>
     </row>
-    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="0" t="s">
         <v>31</v>
       </c>
@@ -1397,7 +1397,7 @@
         <v>8.328</v>
       </c>
     </row>
-    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="0" t="s">
         <v>32</v>
       </c>
@@ -1414,7 +1414,7 @@
         <v>8.328</v>
       </c>
     </row>
-    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="0" t="s">
         <v>33</v>
       </c>
@@ -1431,7 +1431,7 @@
         <v>8.328</v>
       </c>
     </row>
-    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="68" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="0" t="s">
         <v>34</v>
       </c>
@@ -1448,7 +1448,7 @@
         <v>8.328</v>
       </c>
     </row>
-    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="0" t="s">
         <v>35</v>
       </c>
@@ -1465,7 +1465,7 @@
         <v>8.328</v>
       </c>
     </row>
-    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="70" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="0" t="s">
         <v>36</v>
       </c>
@@ -1482,7 +1482,7 @@
         <v>8.328</v>
       </c>
     </row>
-    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="71" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="0" t="s">
         <v>37</v>
       </c>
@@ -1499,7 +1499,7 @@
         <v>8.328</v>
       </c>
     </row>
-    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="72" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="0" t="s">
         <v>38</v>
       </c>
@@ -1516,7 +1516,7 @@
         <v>8.328</v>
       </c>
     </row>
-    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="0" t="s">
         <v>39</v>
       </c>
@@ -1533,7 +1533,7 @@
         <v>8.328</v>
       </c>
     </row>
-    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="74" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="0" t="s">
         <v>40</v>
       </c>
@@ -1550,7 +1550,7 @@
         <v>8.328</v>
       </c>
     </row>
-    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="75" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="0" t="s">
         <v>41</v>
       </c>
@@ -1567,7 +1567,7 @@
         <v>8.328</v>
       </c>
     </row>
-    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="76" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="0" t="s">
         <v>42</v>
       </c>
@@ -1584,7 +1584,7 @@
         <v>8.328</v>
       </c>
     </row>
-    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="77" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="0" t="s">
         <v>43</v>
       </c>
@@ -1601,7 +1601,7 @@
         <v>8.328</v>
       </c>
     </row>
-    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="78" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="0" t="s">
         <v>5</v>
       </c>
@@ -1618,7 +1618,7 @@
         <v>1.969</v>
       </c>
     </row>
-    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="79" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="0" t="s">
         <v>7</v>
       </c>
@@ -1635,7 +1635,7 @@
         <v>1.969</v>
       </c>
     </row>
-    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="80" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="0" t="s">
         <v>8</v>
       </c>
@@ -1643,7 +1643,7 @@
         <v>45</v>
       </c>
       <c r="C80" s="0" t="n">
-        <v>1.969</v>
+        <v>-1.969</v>
       </c>
       <c r="D80" s="0" t="n">
         <v>0.18</v>
@@ -1652,7 +1652,7 @@
         <v>1.969</v>
       </c>
     </row>
-    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="81" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="0" t="s">
         <v>9</v>
       </c>
@@ -1669,7 +1669,7 @@
         <v>1.969</v>
       </c>
     </row>
-    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="82" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="0" t="s">
         <v>10</v>
       </c>
@@ -1686,7 +1686,7 @@
         <v>1.969</v>
       </c>
     </row>
-    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="83" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="0" t="s">
         <v>11</v>
       </c>
@@ -1703,7 +1703,7 @@
         <v>1.969</v>
       </c>
     </row>
-    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="84" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="0" t="s">
         <v>12</v>
       </c>
@@ -1720,7 +1720,7 @@
         <v>1.969</v>
       </c>
     </row>
-    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="85" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="0" t="s">
         <v>13</v>
       </c>
@@ -1737,7 +1737,7 @@
         <v>1.969</v>
       </c>
     </row>
-    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="86" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="0" t="s">
         <v>14</v>
       </c>
@@ -1754,7 +1754,7 @@
         <v>1.969</v>
       </c>
     </row>
-    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="87" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="0" t="s">
         <v>15</v>
       </c>
@@ -1771,7 +1771,7 @@
         <v>1.969</v>
       </c>
     </row>
-    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="88" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="0" t="s">
         <v>16</v>
       </c>
@@ -1788,7 +1788,7 @@
         <v>1.969</v>
       </c>
     </row>
-    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="89" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="0" t="s">
         <v>17</v>
       </c>
@@ -1805,7 +1805,7 @@
         <v>1.969</v>
       </c>
     </row>
-    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="90" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="0" t="s">
         <v>18</v>
       </c>
@@ -1822,7 +1822,7 @@
         <v>1.969</v>
       </c>
     </row>
-    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="91" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="0" t="s">
         <v>19</v>
       </c>
@@ -1839,7 +1839,7 @@
         <v>1.969</v>
       </c>
     </row>
-    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="92" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="0" t="s">
         <v>20</v>
       </c>
@@ -1856,7 +1856,7 @@
         <v>1.969</v>
       </c>
     </row>
-    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="93" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="0" t="s">
         <v>21</v>
       </c>
@@ -1873,7 +1873,7 @@
         <v>1.969</v>
       </c>
     </row>
-    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="94" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="0" t="s">
         <v>22</v>
       </c>
@@ -1890,7 +1890,7 @@
         <v>1.969</v>
       </c>
     </row>
-    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="95" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="0" t="s">
         <v>23</v>
       </c>
@@ -1907,7 +1907,7 @@
         <v>1.969</v>
       </c>
     </row>
-    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="96" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="0" t="s">
         <v>24</v>
       </c>
@@ -1924,7 +1924,7 @@
         <v>1.969</v>
       </c>
     </row>
-    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="97" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="0" t="s">
         <v>25</v>
       </c>
@@ -1941,7 +1941,7 @@
         <v>1.969</v>
       </c>
     </row>
-    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="98" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="0" t="s">
         <v>26</v>
       </c>
@@ -1958,7 +1958,7 @@
         <v>1.969</v>
       </c>
     </row>
-    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="99" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="0" t="s">
         <v>27</v>
       </c>
@@ -1975,7 +1975,7 @@
         <v>1.969</v>
       </c>
     </row>
-    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="100" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="0" t="s">
         <v>28</v>
       </c>
@@ -1992,7 +1992,7 @@
         <v>1.969</v>
       </c>
     </row>
-    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="101" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="0" t="s">
         <v>29</v>
       </c>
@@ -2009,7 +2009,7 @@
         <v>1.969</v>
       </c>
     </row>
-    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="102" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="0" t="s">
         <v>30</v>
       </c>
@@ -2026,7 +2026,7 @@
         <v>1.969</v>
       </c>
     </row>
-    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="103" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="0" t="s">
         <v>31</v>
       </c>
@@ -2043,7 +2043,7 @@
         <v>1.969</v>
       </c>
     </row>
-    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="104" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="0" t="s">
         <v>32</v>
       </c>
@@ -2060,7 +2060,7 @@
         <v>1.969</v>
       </c>
     </row>
-    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="105" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="0" t="s">
         <v>33</v>
       </c>
@@ -2077,7 +2077,7 @@
         <v>1.969</v>
       </c>
     </row>
-    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="106" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="0" t="s">
         <v>34</v>
       </c>
@@ -2094,7 +2094,7 @@
         <v>1.969</v>
       </c>
     </row>
-    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="107" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="0" t="s">
         <v>35</v>
       </c>
@@ -2111,7 +2111,7 @@
         <v>1.969</v>
       </c>
     </row>
-    <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="108" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="0" t="s">
         <v>36</v>
       </c>
@@ -2128,7 +2128,7 @@
         <v>1.969</v>
       </c>
     </row>
-    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="109" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="0" t="s">
         <v>37</v>
       </c>
@@ -2145,7 +2145,7 @@
         <v>1.969</v>
       </c>
     </row>
-    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="110" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="0" t="s">
         <v>38</v>
       </c>
@@ -2162,7 +2162,7 @@
         <v>1.969</v>
       </c>
     </row>
-    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="111" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="0" t="s">
         <v>39</v>
       </c>
@@ -2179,7 +2179,7 @@
         <v>1.969</v>
       </c>
     </row>
-    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="112" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="0" t="s">
         <v>40</v>
       </c>
@@ -2196,7 +2196,7 @@
         <v>1.969</v>
       </c>
     </row>
-    <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="113" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="0" t="s">
         <v>41</v>
       </c>
@@ -2213,7 +2213,7 @@
         <v>1.969</v>
       </c>
     </row>
-    <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="114" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="0" t="s">
         <v>42</v>
       </c>
@@ -2230,7 +2230,7 @@
         <v>1.969</v>
       </c>
     </row>
-    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="115" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="0" t="s">
         <v>43</v>
       </c>
@@ -2247,7 +2247,7 @@
         <v>1.969</v>
       </c>
     </row>
-    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="116" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="0" t="s">
         <v>5</v>
       </c>
@@ -2255,7 +2255,7 @@
         <v>46</v>
       </c>
       <c r="C116" s="0" t="n">
-        <v>-6.82701917999702</v>
+        <v>6.82701917999702</v>
       </c>
       <c r="D116" s="0" t="n">
         <v>0.65</v>
@@ -2264,7 +2264,7 @@
         <v>9.654</v>
       </c>
     </row>
-    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="117" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="0" t="s">
         <v>7</v>
       </c>
@@ -2281,7 +2281,7 @@
         <v>9.654</v>
       </c>
     </row>
-    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="118" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="0" t="s">
         <v>8</v>
       </c>
@@ -2298,7 +2298,7 @@
         <v>9.654</v>
       </c>
     </row>
-    <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="119" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="0" t="s">
         <v>9</v>
       </c>
@@ -2306,7 +2306,7 @@
         <v>46</v>
       </c>
       <c r="C119" s="0" t="n">
-        <v>9.654</v>
+        <v>-9.654</v>
       </c>
       <c r="D119" s="0" t="n">
         <v>0.65</v>
@@ -2315,7 +2315,7 @@
         <v>9.654</v>
       </c>
     </row>
-    <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="120" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="0" t="s">
         <v>10</v>
       </c>
@@ -2332,7 +2332,7 @@
         <v>9.654</v>
       </c>
     </row>
-    <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="121" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="0" t="s">
         <v>11</v>
       </c>
@@ -2349,7 +2349,7 @@
         <v>9.654</v>
       </c>
     </row>
-    <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="122" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="0" t="s">
         <v>12</v>
       </c>
@@ -2366,7 +2366,7 @@
         <v>9.654</v>
       </c>
     </row>
-    <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="123" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="0" t="s">
         <v>13</v>
       </c>
@@ -2383,7 +2383,7 @@
         <v>9.654</v>
       </c>
     </row>
-    <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="124" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="0" t="s">
         <v>14</v>
       </c>
@@ -2400,7 +2400,7 @@
         <v>9.654</v>
       </c>
     </row>
-    <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="125" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="0" t="s">
         <v>15</v>
       </c>
@@ -2417,7 +2417,7 @@
         <v>9.654</v>
       </c>
     </row>
-    <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="126" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="0" t="s">
         <v>16</v>
       </c>
@@ -2434,7 +2434,7 @@
         <v>9.654</v>
       </c>
     </row>
-    <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="127" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="0" t="s">
         <v>17</v>
       </c>
@@ -2451,7 +2451,7 @@
         <v>9.654</v>
       </c>
     </row>
-    <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="128" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="0" t="s">
         <v>18</v>
       </c>
@@ -2468,7 +2468,7 @@
         <v>9.654</v>
       </c>
     </row>
-    <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="129" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="0" t="s">
         <v>19</v>
       </c>
@@ -2485,7 +2485,7 @@
         <v>9.654</v>
       </c>
     </row>
-    <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="130" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="0" t="s">
         <v>20</v>
       </c>
@@ -2502,7 +2502,7 @@
         <v>9.654</v>
       </c>
     </row>
-    <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="131" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="0" t="s">
         <v>21</v>
       </c>
@@ -2519,7 +2519,7 @@
         <v>9.654</v>
       </c>
     </row>
-    <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="132" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="0" t="s">
         <v>22</v>
       </c>
@@ -2536,7 +2536,7 @@
         <v>9.654</v>
       </c>
     </row>
-    <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="133" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A133" s="0" t="s">
         <v>23</v>
       </c>
@@ -2553,7 +2553,7 @@
         <v>9.654</v>
       </c>
     </row>
-    <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="134" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="0" t="s">
         <v>24</v>
       </c>
@@ -2570,7 +2570,7 @@
         <v>9.654</v>
       </c>
     </row>
-    <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="135" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="0" t="s">
         <v>25</v>
       </c>
@@ -2587,7 +2587,7 @@
         <v>9.654</v>
       </c>
     </row>
-    <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="136" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="0" t="s">
         <v>26</v>
       </c>
@@ -2604,7 +2604,7 @@
         <v>9.654</v>
       </c>
     </row>
-    <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="137" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A137" s="0" t="s">
         <v>27</v>
       </c>
@@ -2621,7 +2621,7 @@
         <v>9.654</v>
       </c>
     </row>
-    <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="138" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="0" t="s">
         <v>28</v>
       </c>
@@ -2638,7 +2638,7 @@
         <v>9.654</v>
       </c>
     </row>
-    <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="139" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A139" s="0" t="s">
         <v>29</v>
       </c>
@@ -2655,7 +2655,7 @@
         <v>9.654</v>
       </c>
     </row>
-    <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="140" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A140" s="0" t="s">
         <v>30</v>
       </c>
@@ -2672,7 +2672,7 @@
         <v>9.654</v>
       </c>
     </row>
-    <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="141" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A141" s="0" t="s">
         <v>31</v>
       </c>
@@ -2689,7 +2689,7 @@
         <v>9.654</v>
       </c>
     </row>
-    <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="142" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A142" s="0" t="s">
         <v>32</v>
       </c>
@@ -2706,7 +2706,7 @@
         <v>9.654</v>
       </c>
     </row>
-    <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="143" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A143" s="0" t="s">
         <v>33</v>
       </c>
@@ -2723,7 +2723,7 @@
         <v>9.654</v>
       </c>
     </row>
-    <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="144" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A144" s="0" t="s">
         <v>34</v>
       </c>
@@ -2740,7 +2740,7 @@
         <v>9.654</v>
       </c>
     </row>
-    <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="145" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A145" s="0" t="s">
         <v>35</v>
       </c>
@@ -2757,7 +2757,7 @@
         <v>9.654</v>
       </c>
     </row>
-    <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="146" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A146" s="0" t="s">
         <v>36</v>
       </c>
@@ -2774,7 +2774,7 @@
         <v>9.654</v>
       </c>
     </row>
-    <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="147" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A147" s="0" t="s">
         <v>37</v>
       </c>
@@ -2791,7 +2791,7 @@
         <v>9.654</v>
       </c>
     </row>
-    <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="148" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A148" s="0" t="s">
         <v>38</v>
       </c>
@@ -2808,7 +2808,7 @@
         <v>9.654</v>
       </c>
     </row>
-    <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="149" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A149" s="0" t="s">
         <v>39</v>
       </c>
@@ -2825,7 +2825,7 @@
         <v>9.654</v>
       </c>
     </row>
-    <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="150" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A150" s="0" t="s">
         <v>40</v>
       </c>
@@ -2842,7 +2842,7 @@
         <v>9.654</v>
       </c>
     </row>
-    <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="151" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A151" s="0" t="s">
         <v>41</v>
       </c>
@@ -2859,7 +2859,7 @@
         <v>9.654</v>
       </c>
     </row>
-    <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="152" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A152" s="0" t="s">
         <v>42</v>
       </c>
@@ -2876,7 +2876,7 @@
         <v>9.654</v>
       </c>
     </row>
-    <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="153" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A153" s="0" t="s">
         <v>43</v>
       </c>
@@ -2893,7 +2893,7 @@
         <v>9.654</v>
       </c>
     </row>
-    <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="154" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A154" s="0" t="s">
         <v>5</v>
       </c>
@@ -2901,7 +2901,7 @@
         <v>47</v>
       </c>
       <c r="C154" s="0" t="n">
-        <v>-0.5970002640036</v>
+        <v>0.5970002640036</v>
       </c>
       <c r="D154" s="0" t="n">
         <v>0.49</v>
@@ -2910,7 +2910,7 @@
         <v>4.9448</v>
       </c>
     </row>
-    <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="155" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A155" s="0" t="s">
         <v>7</v>
       </c>
@@ -2927,7 +2927,7 @@
         <v>4.9448</v>
       </c>
     </row>
-    <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="156" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A156" s="0" t="s">
         <v>8</v>
       </c>
@@ -2944,7 +2944,7 @@
         <v>4.9448</v>
       </c>
     </row>
-    <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="157" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A157" s="0" t="s">
         <v>9</v>
       </c>
@@ -2961,7 +2961,7 @@
         <v>4.9448</v>
       </c>
     </row>
-    <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="158" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A158" s="0" t="s">
         <v>10</v>
       </c>
@@ -2969,7 +2969,7 @@
         <v>47</v>
       </c>
       <c r="C158" s="0" t="n">
-        <v>4.94483364720653</v>
+        <v>-4.94483364720653</v>
       </c>
       <c r="D158" s="0" t="n">
         <v>0.49</v>
@@ -2978,7 +2978,7 @@
         <v>4.9448</v>
       </c>
     </row>
-    <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="159" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A159" s="0" t="s">
         <v>11</v>
       </c>
@@ -2995,7 +2995,7 @@
         <v>4.9448</v>
       </c>
     </row>
-    <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="160" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A160" s="0" t="s">
         <v>12</v>
       </c>
@@ -3012,7 +3012,7 @@
         <v>4.9448</v>
       </c>
     </row>
-    <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="161" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A161" s="0" t="s">
         <v>13</v>
       </c>
@@ -3029,7 +3029,7 @@
         <v>4.9448</v>
       </c>
     </row>
-    <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="162" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A162" s="0" t="s">
         <v>14</v>
       </c>
@@ -3046,7 +3046,7 @@
         <v>4.9448</v>
       </c>
     </row>
-    <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="163" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A163" s="0" t="s">
         <v>15</v>
       </c>
@@ -3063,7 +3063,7 @@
         <v>4.9448</v>
       </c>
     </row>
-    <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="164" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A164" s="0" t="s">
         <v>16</v>
       </c>
@@ -3080,7 +3080,7 @@
         <v>4.9448</v>
       </c>
     </row>
-    <row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="165" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A165" s="0" t="s">
         <v>17</v>
       </c>
@@ -3097,7 +3097,7 @@
         <v>4.9448</v>
       </c>
     </row>
-    <row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="166" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A166" s="0" t="s">
         <v>18</v>
       </c>
@@ -3114,7 +3114,7 @@
         <v>4.9448</v>
       </c>
     </row>
-    <row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="167" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A167" s="0" t="s">
         <v>19</v>
       </c>
@@ -3131,7 +3131,7 @@
         <v>4.9448</v>
       </c>
     </row>
-    <row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="168" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A168" s="0" t="s">
         <v>20</v>
       </c>
@@ -3148,7 +3148,7 @@
         <v>4.9448</v>
       </c>
     </row>
-    <row r="169" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="169" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A169" s="0" t="s">
         <v>21</v>
       </c>
@@ -3165,7 +3165,7 @@
         <v>4.9448</v>
       </c>
     </row>
-    <row r="170" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="170" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A170" s="0" t="s">
         <v>22</v>
       </c>
@@ -3182,7 +3182,7 @@
         <v>4.9448</v>
       </c>
     </row>
-    <row r="171" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="171" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A171" s="0" t="s">
         <v>23</v>
       </c>
@@ -3199,7 +3199,7 @@
         <v>4.9448</v>
       </c>
     </row>
-    <row r="172" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="172" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A172" s="0" t="s">
         <v>24</v>
       </c>
@@ -3216,7 +3216,7 @@
         <v>4.9448</v>
       </c>
     </row>
-    <row r="173" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="173" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A173" s="0" t="s">
         <v>25</v>
       </c>
@@ -3233,7 +3233,7 @@
         <v>4.9448</v>
       </c>
     </row>
-    <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="174" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A174" s="0" t="s">
         <v>26</v>
       </c>
@@ -3250,7 +3250,7 @@
         <v>4.9448</v>
       </c>
     </row>
-    <row r="175" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="175" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A175" s="0" t="s">
         <v>27</v>
       </c>
@@ -3267,7 +3267,7 @@
         <v>4.9448</v>
       </c>
     </row>
-    <row r="176" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="176" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A176" s="0" t="s">
         <v>28</v>
       </c>
@@ -3284,7 +3284,7 @@
         <v>4.9448</v>
       </c>
     </row>
-    <row r="177" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="177" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A177" s="0" t="s">
         <v>29</v>
       </c>
@@ -3301,7 +3301,7 @@
         <v>4.9448</v>
       </c>
     </row>
-    <row r="178" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="178" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A178" s="0" t="s">
         <v>30</v>
       </c>
@@ -3318,7 +3318,7 @@
         <v>4.9448</v>
       </c>
     </row>
-    <row r="179" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="179" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A179" s="0" t="s">
         <v>31</v>
       </c>
@@ -3335,7 +3335,7 @@
         <v>4.9448</v>
       </c>
     </row>
-    <row r="180" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="180" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A180" s="0" t="s">
         <v>32</v>
       </c>
@@ -3352,7 +3352,7 @@
         <v>4.9448</v>
       </c>
     </row>
-    <row r="181" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="181" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A181" s="0" t="s">
         <v>33</v>
       </c>
@@ -3369,7 +3369,7 @@
         <v>4.9448</v>
       </c>
     </row>
-    <row r="182" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="182" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A182" s="0" t="s">
         <v>34</v>
       </c>
@@ -3386,7 +3386,7 @@
         <v>4.9448</v>
       </c>
     </row>
-    <row r="183" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="183" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A183" s="0" t="s">
         <v>35</v>
       </c>
@@ -3403,7 +3403,7 @@
         <v>4.9448</v>
       </c>
     </row>
-    <row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="184" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A184" s="0" t="s">
         <v>36</v>
       </c>
@@ -3420,7 +3420,7 @@
         <v>4.9448</v>
       </c>
     </row>
-    <row r="185" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="185" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A185" s="0" t="s">
         <v>37</v>
       </c>
@@ -3437,7 +3437,7 @@
         <v>4.9448</v>
       </c>
     </row>
-    <row r="186" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="186" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A186" s="0" t="s">
         <v>38</v>
       </c>
@@ -3454,7 +3454,7 @@
         <v>4.9448</v>
       </c>
     </row>
-    <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="187" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A187" s="0" t="s">
         <v>39</v>
       </c>
@@ -3471,7 +3471,7 @@
         <v>4.9448</v>
       </c>
     </row>
-    <row r="188" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="188" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A188" s="0" t="s">
         <v>40</v>
       </c>
@@ -3488,7 +3488,7 @@
         <v>4.9448</v>
       </c>
     </row>
-    <row r="189" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="189" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A189" s="0" t="s">
         <v>41</v>
       </c>
@@ -3505,7 +3505,7 @@
         <v>4.9448</v>
       </c>
     </row>
-    <row r="190" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="190" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A190" s="0" t="s">
         <v>42</v>
       </c>
@@ -3522,7 +3522,7 @@
         <v>4.9448</v>
       </c>
     </row>
-    <row r="191" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="191" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A191" s="0" t="s">
         <v>43</v>
       </c>
@@ -3539,7 +3539,7 @@
         <v>4.9448</v>
       </c>
     </row>
-    <row r="192" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="192" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A192" s="0" t="s">
         <v>5</v>
       </c>
@@ -3547,7 +3547,7 @@
         <v>48</v>
       </c>
       <c r="C192" s="0" t="n">
-        <v>-5.00398239363803</v>
+        <v>5.00398239363803</v>
       </c>
       <c r="D192" s="0" t="n">
         <v>0.59</v>
@@ -3556,7 +3556,7 @@
         <v>7.2839</v>
       </c>
     </row>
-    <row r="193" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="193" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A193" s="0" t="s">
         <v>7</v>
       </c>
@@ -3573,7 +3573,7 @@
         <v>7.2839</v>
       </c>
     </row>
-    <row r="194" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="194" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A194" s="0" t="s">
         <v>8</v>
       </c>
@@ -3590,7 +3590,7 @@
         <v>7.2839</v>
       </c>
     </row>
-    <row r="195" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="195" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A195" s="0" t="s">
         <v>9</v>
       </c>
@@ -3607,7 +3607,7 @@
         <v>7.2839</v>
       </c>
     </row>
-    <row r="196" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="196" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A196" s="0" t="s">
         <v>10</v>
       </c>
@@ -3624,7 +3624,7 @@
         <v>7.2839</v>
       </c>
     </row>
-    <row r="197" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="197" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A197" s="0" t="s">
         <v>11</v>
       </c>
@@ -3632,7 +3632,7 @@
         <v>48</v>
       </c>
       <c r="C197" s="0" t="n">
-        <v>7.28392319195215</v>
+        <v>-7.28392319195215</v>
       </c>
       <c r="D197" s="0" t="n">
         <v>0.59</v>
@@ -3641,7 +3641,7 @@
         <v>7.2839</v>
       </c>
     </row>
-    <row r="198" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="198" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A198" s="0" t="s">
         <v>12</v>
       </c>
@@ -3658,7 +3658,7 @@
         <v>7.2839</v>
       </c>
     </row>
-    <row r="199" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="199" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A199" s="0" t="s">
         <v>13</v>
       </c>
@@ -3675,7 +3675,7 @@
         <v>7.2839</v>
       </c>
     </row>
-    <row r="200" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="200" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A200" s="0" t="s">
         <v>14</v>
       </c>
@@ -3692,7 +3692,7 @@
         <v>7.2839</v>
       </c>
     </row>
-    <row r="201" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="201" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A201" s="0" t="s">
         <v>15</v>
       </c>
@@ -3709,7 +3709,7 @@
         <v>7.2839</v>
       </c>
     </row>
-    <row r="202" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="202" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A202" s="0" t="s">
         <v>16</v>
       </c>
@@ -3726,7 +3726,7 @@
         <v>7.2839</v>
       </c>
     </row>
-    <row r="203" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="203" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A203" s="0" t="s">
         <v>17</v>
       </c>
@@ -3743,7 +3743,7 @@
         <v>7.2839</v>
       </c>
     </row>
-    <row r="204" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="204" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A204" s="0" t="s">
         <v>18</v>
       </c>
@@ -3760,7 +3760,7 @@
         <v>7.2839</v>
       </c>
     </row>
-    <row r="205" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="205" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A205" s="0" t="s">
         <v>19</v>
       </c>
@@ -3777,7 +3777,7 @@
         <v>7.2839</v>
       </c>
     </row>
-    <row r="206" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="206" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A206" s="0" t="s">
         <v>20</v>
       </c>
@@ -3794,7 +3794,7 @@
         <v>7.2839</v>
       </c>
     </row>
-    <row r="207" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="207" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A207" s="0" t="s">
         <v>21</v>
       </c>
@@ -3811,7 +3811,7 @@
         <v>7.2839</v>
       </c>
     </row>
-    <row r="208" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="208" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A208" s="0" t="s">
         <v>22</v>
       </c>
@@ -3828,7 +3828,7 @@
         <v>7.2839</v>
       </c>
     </row>
-    <row r="209" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="209" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A209" s="0" t="s">
         <v>23</v>
       </c>
@@ -3845,7 +3845,7 @@
         <v>7.2839</v>
       </c>
     </row>
-    <row r="210" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="210" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A210" s="0" t="s">
         <v>24</v>
       </c>
@@ -3862,7 +3862,7 @@
         <v>7.2839</v>
       </c>
     </row>
-    <row r="211" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="211" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A211" s="0" t="s">
         <v>25</v>
       </c>
@@ -3879,7 +3879,7 @@
         <v>7.2839</v>
       </c>
     </row>
-    <row r="212" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="212" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A212" s="0" t="s">
         <v>26</v>
       </c>
@@ -3896,7 +3896,7 @@
         <v>7.2839</v>
       </c>
     </row>
-    <row r="213" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="213" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A213" s="0" t="s">
         <v>27</v>
       </c>
@@ -3913,7 +3913,7 @@
         <v>7.2839</v>
       </c>
     </row>
-    <row r="214" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="214" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A214" s="0" t="s">
         <v>28</v>
       </c>
@@ -3930,7 +3930,7 @@
         <v>7.2839</v>
       </c>
     </row>
-    <row r="215" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="215" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A215" s="0" t="s">
         <v>29</v>
       </c>
@@ -3947,7 +3947,7 @@
         <v>7.2839</v>
       </c>
     </row>
-    <row r="216" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="216" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A216" s="0" t="s">
         <v>30</v>
       </c>
@@ -3964,7 +3964,7 @@
         <v>7.2839</v>
       </c>
     </row>
-    <row r="217" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="217" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A217" s="0" t="s">
         <v>31</v>
       </c>
@@ -3981,7 +3981,7 @@
         <v>7.2839</v>
       </c>
     </row>
-    <row r="218" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="218" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A218" s="0" t="s">
         <v>32</v>
       </c>
@@ -3998,7 +3998,7 @@
         <v>7.2839</v>
       </c>
     </row>
-    <row r="219" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="219" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A219" s="0" t="s">
         <v>33</v>
       </c>
@@ -4015,7 +4015,7 @@
         <v>7.2839</v>
       </c>
     </row>
-    <row r="220" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="220" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A220" s="0" t="s">
         <v>34</v>
       </c>
@@ -4032,7 +4032,7 @@
         <v>7.2839</v>
       </c>
     </row>
-    <row r="221" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="221" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A221" s="0" t="s">
         <v>35</v>
       </c>
@@ -4049,7 +4049,7 @@
         <v>7.2839</v>
       </c>
     </row>
-    <row r="222" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="222" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A222" s="0" t="s">
         <v>36</v>
       </c>
@@ -4066,7 +4066,7 @@
         <v>7.2839</v>
       </c>
     </row>
-    <row r="223" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="223" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A223" s="0" t="s">
         <v>37</v>
       </c>
@@ -4083,7 +4083,7 @@
         <v>7.2839</v>
       </c>
     </row>
-    <row r="224" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="224" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A224" s="0" t="s">
         <v>38</v>
       </c>
@@ -4100,7 +4100,7 @@
         <v>7.2839</v>
       </c>
     </row>
-    <row r="225" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="225" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A225" s="0" t="s">
         <v>39</v>
       </c>
@@ -4117,7 +4117,7 @@
         <v>7.2839</v>
       </c>
     </row>
-    <row r="226" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="226" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A226" s="0" t="s">
         <v>40</v>
       </c>
@@ -4134,7 +4134,7 @@
         <v>7.2839</v>
       </c>
     </row>
-    <row r="227" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="227" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A227" s="0" t="s">
         <v>41</v>
       </c>
@@ -4151,7 +4151,7 @@
         <v>7.2839</v>
       </c>
     </row>
-    <row r="228" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="228" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A228" s="0" t="s">
         <v>42</v>
       </c>
@@ -4168,7 +4168,7 @@
         <v>7.2839</v>
       </c>
     </row>
-    <row r="229" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="229" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A229" s="0" t="s">
         <v>43</v>
       </c>
@@ -4185,7 +4185,7 @@
         <v>7.2839</v>
       </c>
     </row>
-    <row r="230" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="230" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A230" s="0" t="s">
         <v>5</v>
       </c>
@@ -4193,7 +4193,7 @@
         <v>49</v>
       </c>
       <c r="C230" s="0" t="n">
-        <v>-11.9139097200115</v>
+        <v>11.9139097200115</v>
       </c>
       <c r="D230" s="0" t="n">
         <v>0.39</v>
@@ -4202,7 +4202,7 @@
         <v>26.714</v>
       </c>
     </row>
-    <row r="231" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="231" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A231" s="0" t="s">
         <v>7</v>
       </c>
@@ -4219,7 +4219,7 @@
         <v>26.714</v>
       </c>
     </row>
-    <row r="232" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="232" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A232" s="0" t="s">
         <v>8</v>
       </c>
@@ -4236,7 +4236,7 @@
         <v>26.714</v>
       </c>
     </row>
-    <row r="233" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="233" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A233" s="0" t="s">
         <v>9</v>
       </c>
@@ -4253,7 +4253,7 @@
         <v>26.714</v>
       </c>
     </row>
-    <row r="234" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="234" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A234" s="0" t="s">
         <v>10</v>
       </c>
@@ -4270,7 +4270,7 @@
         <v>26.714</v>
       </c>
     </row>
-    <row r="235" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="235" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A235" s="0" t="s">
         <v>11</v>
       </c>
@@ -4287,7 +4287,7 @@
         <v>26.714</v>
       </c>
     </row>
-    <row r="236" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="236" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A236" s="0" t="s">
         <v>12</v>
       </c>
@@ -4295,7 +4295,7 @@
         <v>49</v>
       </c>
       <c r="C236" s="0" t="n">
-        <v>26.714</v>
+        <v>-26.714</v>
       </c>
       <c r="D236" s="0" t="n">
         <v>0.39</v>
@@ -4304,7 +4304,7 @@
         <v>26.714</v>
       </c>
     </row>
-    <row r="237" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="237" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A237" s="0" t="s">
         <v>13</v>
       </c>
@@ -4321,7 +4321,7 @@
         <v>26.714</v>
       </c>
     </row>
-    <row r="238" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="238" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A238" s="0" t="s">
         <v>14</v>
       </c>
@@ -4338,7 +4338,7 @@
         <v>26.714</v>
       </c>
     </row>
-    <row r="239" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="239" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A239" s="0" t="s">
         <v>15</v>
       </c>
@@ -4346,7 +4346,7 @@
         <v>49</v>
       </c>
       <c r="C239" s="0" t="n">
-        <v>1.15701005397392</v>
+        <v>-1.15701005397392</v>
       </c>
       <c r="D239" s="0" t="n">
         <v>0.39</v>
@@ -4355,7 +4355,7 @@
         <v>26.714</v>
       </c>
     </row>
-    <row r="240" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="240" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A240" s="0" t="s">
         <v>16</v>
       </c>
@@ -4372,7 +4372,7 @@
         <v>26.714</v>
       </c>
     </row>
-    <row r="241" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="241" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A241" s="0" t="s">
         <v>17</v>
       </c>
@@ -4389,7 +4389,7 @@
         <v>26.714</v>
       </c>
     </row>
-    <row r="242" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="242" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A242" s="0" t="s">
         <v>18</v>
       </c>
@@ -4406,7 +4406,7 @@
         <v>26.714</v>
       </c>
     </row>
-    <row r="243" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="243" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A243" s="0" t="s">
         <v>19</v>
       </c>
@@ -4423,7 +4423,7 @@
         <v>26.714</v>
       </c>
     </row>
-    <row r="244" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="244" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A244" s="0" t="s">
         <v>20</v>
       </c>
@@ -4440,7 +4440,7 @@
         <v>26.714</v>
       </c>
     </row>
-    <row r="245" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="245" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A245" s="0" t="s">
         <v>21</v>
       </c>
@@ -4457,7 +4457,7 @@
         <v>26.714</v>
       </c>
     </row>
-    <row r="246" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="246" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A246" s="0" t="s">
         <v>22</v>
       </c>
@@ -4474,7 +4474,7 @@
         <v>26.714</v>
       </c>
     </row>
-    <row r="247" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="247" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A247" s="0" t="s">
         <v>23</v>
       </c>
@@ -4491,7 +4491,7 @@
         <v>26.714</v>
       </c>
     </row>
-    <row r="248" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="248" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A248" s="0" t="s">
         <v>24</v>
       </c>
@@ -4508,7 +4508,7 @@
         <v>26.714</v>
       </c>
     </row>
-    <row r="249" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="249" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A249" s="0" t="s">
         <v>25</v>
       </c>
@@ -4525,7 +4525,7 @@
         <v>26.714</v>
       </c>
     </row>
-    <row r="250" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="250" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A250" s="0" t="s">
         <v>26</v>
       </c>
@@ -4542,7 +4542,7 @@
         <v>26.714</v>
       </c>
     </row>
-    <row r="251" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="251" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A251" s="0" t="s">
         <v>27</v>
       </c>
@@ -4559,7 +4559,7 @@
         <v>26.714</v>
       </c>
     </row>
-    <row r="252" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="252" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A252" s="0" t="s">
         <v>28</v>
       </c>
@@ -4576,7 +4576,7 @@
         <v>26.714</v>
       </c>
     </row>
-    <row r="253" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="253" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A253" s="0" t="s">
         <v>29</v>
       </c>
@@ -4593,7 +4593,7 @@
         <v>26.714</v>
       </c>
     </row>
-    <row r="254" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="254" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A254" s="0" t="s">
         <v>30</v>
       </c>
@@ -4610,7 +4610,7 @@
         <v>26.714</v>
       </c>
     </row>
-    <row r="255" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="255" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A255" s="0" t="s">
         <v>31</v>
       </c>
@@ -4627,7 +4627,7 @@
         <v>26.714</v>
       </c>
     </row>
-    <row r="256" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="256" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A256" s="0" t="s">
         <v>32</v>
       </c>
@@ -4644,7 +4644,7 @@
         <v>26.714</v>
       </c>
     </row>
-    <row r="257" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="257" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A257" s="0" t="s">
         <v>33</v>
       </c>
@@ -4661,7 +4661,7 @@
         <v>26.714</v>
       </c>
     </row>
-    <row r="258" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="258" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A258" s="0" t="s">
         <v>34</v>
       </c>
@@ -4678,7 +4678,7 @@
         <v>26.714</v>
       </c>
     </row>
-    <row r="259" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="259" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A259" s="0" t="s">
         <v>35</v>
       </c>
@@ -4695,7 +4695,7 @@
         <v>26.714</v>
       </c>
     </row>
-    <row r="260" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="260" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A260" s="0" t="s">
         <v>36</v>
       </c>
@@ -4712,7 +4712,7 @@
         <v>26.714</v>
       </c>
     </row>
-    <row r="261" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="261" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A261" s="0" t="s">
         <v>37</v>
       </c>
@@ -4729,7 +4729,7 @@
         <v>26.714</v>
       </c>
     </row>
-    <row r="262" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="262" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A262" s="0" t="s">
         <v>38</v>
       </c>
@@ -4746,7 +4746,7 @@
         <v>26.714</v>
       </c>
     </row>
-    <row r="263" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="263" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A263" s="0" t="s">
         <v>39</v>
       </c>
@@ -4763,7 +4763,7 @@
         <v>26.714</v>
       </c>
     </row>
-    <row r="264" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="264" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A264" s="0" t="s">
         <v>40</v>
       </c>
@@ -4780,7 +4780,7 @@
         <v>26.714</v>
       </c>
     </row>
-    <row r="265" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="265" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A265" s="0" t="s">
         <v>41</v>
       </c>
@@ -4797,7 +4797,7 @@
         <v>26.714</v>
       </c>
     </row>
-    <row r="266" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="266" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A266" s="0" t="s">
         <v>42</v>
       </c>
@@ -4814,7 +4814,7 @@
         <v>26.714</v>
       </c>
     </row>
-    <row r="267" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="267" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A267" s="0" t="s">
         <v>43</v>
       </c>
@@ -4831,7 +4831,7 @@
         <v>26.714</v>
       </c>
     </row>
-    <row r="268" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="268" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A268" s="0" t="s">
         <v>5</v>
       </c>
@@ -4839,7 +4839,7 @@
         <v>50</v>
       </c>
       <c r="C268" s="0" t="n">
-        <v>-3.32097367999354</v>
+        <v>3.32097367999354</v>
       </c>
       <c r="D268" s="0" t="n">
         <v>0.51</v>
@@ -4848,7 +4848,7 @@
         <v>15.902</v>
       </c>
     </row>
-    <row r="269" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="269" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A269" s="0" t="s">
         <v>7</v>
       </c>
@@ -4865,7 +4865,7 @@
         <v>15.902</v>
       </c>
     </row>
-    <row r="270" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="270" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A270" s="0" t="s">
         <v>8</v>
       </c>
@@ -4882,7 +4882,7 @@
         <v>15.902</v>
       </c>
     </row>
-    <row r="271" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="271" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A271" s="0" t="s">
         <v>9</v>
       </c>
@@ -4899,7 +4899,7 @@
         <v>15.902</v>
       </c>
     </row>
-    <row r="272" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="272" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A272" s="0" t="s">
         <v>10</v>
       </c>
@@ -4916,7 +4916,7 @@
         <v>15.902</v>
       </c>
     </row>
-    <row r="273" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="273" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A273" s="0" t="s">
         <v>11</v>
       </c>
@@ -4933,7 +4933,7 @@
         <v>15.902</v>
       </c>
     </row>
-    <row r="274" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="274" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A274" s="0" t="s">
         <v>12</v>
       </c>
@@ -4950,7 +4950,7 @@
         <v>15.902</v>
       </c>
     </row>
-    <row r="275" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="275" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A275" s="0" t="s">
         <v>13</v>
       </c>
@@ -4958,7 +4958,7 @@
         <v>50</v>
       </c>
       <c r="C275" s="0" t="n">
-        <v>15.902</v>
+        <v>-15.902</v>
       </c>
       <c r="D275" s="0" t="n">
         <v>0.51</v>
@@ -4967,7 +4967,7 @@
         <v>15.902</v>
       </c>
     </row>
-    <row r="276" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="276" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A276" s="0" t="s">
         <v>14</v>
       </c>
@@ -4975,7 +4975,7 @@
         <v>50</v>
       </c>
       <c r="C276" s="0" t="n">
-        <v>1.13999847799564</v>
+        <v>-1.13999847799564</v>
       </c>
       <c r="D276" s="0" t="n">
         <v>0.51</v>
@@ -4984,7 +4984,7 @@
         <v>15.902</v>
       </c>
     </row>
-    <row r="277" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="277" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A277" s="0" t="s">
         <v>15</v>
       </c>
@@ -5001,7 +5001,7 @@
         <v>15.902</v>
       </c>
     </row>
-    <row r="278" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="278" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A278" s="0" t="s">
         <v>16</v>
       </c>
@@ -5018,7 +5018,7 @@
         <v>15.902</v>
       </c>
     </row>
-    <row r="279" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="279" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A279" s="0" t="s">
         <v>17</v>
       </c>
@@ -5035,7 +5035,7 @@
         <v>15.902</v>
       </c>
     </row>
-    <row r="280" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="280" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A280" s="0" t="s">
         <v>18</v>
       </c>
@@ -5052,7 +5052,7 @@
         <v>15.902</v>
       </c>
     </row>
-    <row r="281" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="281" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A281" s="0" t="s">
         <v>19</v>
       </c>
@@ -5069,7 +5069,7 @@
         <v>15.902</v>
       </c>
     </row>
-    <row r="282" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="282" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A282" s="0" t="s">
         <v>20</v>
       </c>
@@ -5086,7 +5086,7 @@
         <v>15.902</v>
       </c>
     </row>
-    <row r="283" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="283" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A283" s="0" t="s">
         <v>21</v>
       </c>
@@ -5103,7 +5103,7 @@
         <v>15.902</v>
       </c>
     </row>
-    <row r="284" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="284" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A284" s="0" t="s">
         <v>22</v>
       </c>
@@ -5120,7 +5120,7 @@
         <v>15.902</v>
       </c>
     </row>
-    <row r="285" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="285" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A285" s="0" t="s">
         <v>23</v>
       </c>
@@ -5137,7 +5137,7 @@
         <v>15.902</v>
       </c>
     </row>
-    <row r="286" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="286" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A286" s="0" t="s">
         <v>24</v>
       </c>
@@ -5154,7 +5154,7 @@
         <v>15.902</v>
       </c>
     </row>
-    <row r="287" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="287" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A287" s="0" t="s">
         <v>25</v>
       </c>
@@ -5171,7 +5171,7 @@
         <v>15.902</v>
       </c>
     </row>
-    <row r="288" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="288" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A288" s="0" t="s">
         <v>26</v>
       </c>
@@ -5188,7 +5188,7 @@
         <v>15.902</v>
       </c>
     </row>
-    <row r="289" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="289" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A289" s="0" t="s">
         <v>27</v>
       </c>
@@ -5205,7 +5205,7 @@
         <v>15.902</v>
       </c>
     </row>
-    <row r="290" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="290" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A290" s="0" t="s">
         <v>28</v>
       </c>
@@ -5222,7 +5222,7 @@
         <v>15.902</v>
       </c>
     </row>
-    <row r="291" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="291" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A291" s="0" t="s">
         <v>29</v>
       </c>
@@ -5239,7 +5239,7 @@
         <v>15.902</v>
       </c>
     </row>
-    <row r="292" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="292" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A292" s="0" t="s">
         <v>30</v>
       </c>
@@ -5256,7 +5256,7 @@
         <v>15.902</v>
       </c>
     </row>
-    <row r="293" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="293" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A293" s="0" t="s">
         <v>31</v>
       </c>
@@ -5273,7 +5273,7 @@
         <v>15.902</v>
       </c>
     </row>
-    <row r="294" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="294" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A294" s="0" t="s">
         <v>32</v>
       </c>
@@ -5290,7 +5290,7 @@
         <v>15.902</v>
       </c>
     </row>
-    <row r="295" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="295" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A295" s="0" t="s">
         <v>33</v>
       </c>
@@ -5307,7 +5307,7 @@
         <v>15.902</v>
       </c>
     </row>
-    <row r="296" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="296" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A296" s="0" t="s">
         <v>34</v>
       </c>
@@ -5324,7 +5324,7 @@
         <v>15.902</v>
       </c>
     </row>
-    <row r="297" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="297" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A297" s="0" t="s">
         <v>35</v>
       </c>
@@ -5341,7 +5341,7 @@
         <v>15.902</v>
       </c>
     </row>
-    <row r="298" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="298" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A298" s="0" t="s">
         <v>36</v>
       </c>
@@ -5358,7 +5358,7 @@
         <v>15.902</v>
       </c>
     </row>
-    <row r="299" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="299" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A299" s="0" t="s">
         <v>37</v>
       </c>
@@ -5375,7 +5375,7 @@
         <v>15.902</v>
       </c>
     </row>
-    <row r="300" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="300" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A300" s="0" t="s">
         <v>38</v>
       </c>
@@ -5392,7 +5392,7 @@
         <v>15.902</v>
       </c>
     </row>
-    <row r="301" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="301" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A301" s="0" t="s">
         <v>39</v>
       </c>
@@ -5409,7 +5409,7 @@
         <v>15.902</v>
       </c>
     </row>
-    <row r="302" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="302" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A302" s="0" t="s">
         <v>40</v>
       </c>
@@ -5426,7 +5426,7 @@
         <v>15.902</v>
       </c>
     </row>
-    <row r="303" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="303" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A303" s="0" t="s">
         <v>41</v>
       </c>
@@ -5443,7 +5443,7 @@
         <v>15.902</v>
       </c>
     </row>
-    <row r="304" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="304" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A304" s="0" t="s">
         <v>42</v>
       </c>
@@ -5460,7 +5460,7 @@
         <v>15.902</v>
       </c>
     </row>
-    <row r="305" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="305" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A305" s="0" t="s">
         <v>43</v>
       </c>

</xml_diff>